<commit_message>
Data Analysis | Creation of plots
</commit_message>
<xml_diff>
--- a/data_analysis/data_analysis.xlsx
+++ b/data_analysis/data_analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\river\OneDrive - Radboud Universiteit\Documenten\GitHub\thesis_face_gesture_project\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B59CE78-7E82-4C2D-A76C-AB64261757C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3640C26-6D14-46A2-AC2A-5B70A2D99B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Python" sheetId="3" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="113">
   <si>
     <t>Marca temporal</t>
   </si>
@@ -362,6 +362,21 @@
   <si>
     <t>System B Accuracy</t>
   </si>
+  <si>
+    <t>ID_012</t>
+  </si>
+  <si>
+    <t>ID_013</t>
+  </si>
+  <si>
+    <t>ID_014</t>
+  </si>
+  <si>
+    <t>ID_015</t>
+  </si>
+  <si>
+    <t>ID_016</t>
+  </si>
 </sst>
 </file>
 
@@ -369,9 +384,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
-    <numFmt numFmtId="171" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -405,6 +420,28 @@
     <font>
       <sz val="8"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -608,7 +645,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -666,12 +703,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="171" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1031,7 +1072,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>91</v>
       </c>
@@ -1108,7 +1149,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>92</v>
       </c>
@@ -1185,7 +1226,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>93</v>
       </c>
@@ -1262,7 +1303,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>94</v>
       </c>
@@ -1339,7 +1380,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>95</v>
       </c>
@@ -1416,7 +1457,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>96</v>
       </c>
@@ -1430,7 +1471,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F7" s="13">
         <v>1</v>
@@ -1493,7 +1534,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>97</v>
       </c>
@@ -1570,7 +1611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>98</v>
       </c>
@@ -1647,7 +1688,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>99</v>
       </c>
@@ -1724,7 +1765,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>100</v>
       </c>
@@ -1801,7 +1842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>101</v>
       </c>
@@ -1877,32 +1918,315 @@
       <c r="Y12" s="20">
         <v>2</v>
       </c>
-    </row>
-    <row r="16" spans="1:31" ht="13" x14ac:dyDescent="0.3">
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="21"/>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="21"/>
-      <c r="O16" s="21"/>
-      <c r="P16" s="21"/>
-      <c r="Q16" s="21"/>
-      <c r="R16" s="22"/>
-      <c r="S16" s="22"/>
-      <c r="T16" s="21"/>
-      <c r="U16" s="21"/>
-      <c r="V16" s="21"/>
-      <c r="W16" s="21"/>
-      <c r="X16" s="21"/>
-      <c r="Y16" s="21"/>
+      <c r="Z12" s="28"/>
+    </row>
+    <row r="13" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="B13" s="13">
+        <v>3</v>
+      </c>
+      <c r="C13">
+        <v>3</v>
+      </c>
+      <c r="D13" s="13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>2</v>
+      </c>
+      <c r="F13" s="13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>2</v>
+      </c>
+      <c r="H13" s="13">
+        <v>2</v>
+      </c>
+      <c r="I13">
+        <v>2</v>
+      </c>
+      <c r="J13" s="13">
+        <v>2</v>
+      </c>
+      <c r="K13">
+        <v>3</v>
+      </c>
+      <c r="L13" s="13">
+        <v>3</v>
+      </c>
+      <c r="M13">
+        <v>4</v>
+      </c>
+      <c r="N13" s="13">
+        <v>2</v>
+      </c>
+      <c r="O13">
+        <v>3</v>
+      </c>
+      <c r="P13" s="13">
+        <v>4</v>
+      </c>
+      <c r="Q13">
+        <v>4</v>
+      </c>
+      <c r="R13" s="13">
+        <v>4</v>
+      </c>
+      <c r="S13">
+        <v>4</v>
+      </c>
+      <c r="T13" s="13">
+        <v>2</v>
+      </c>
+      <c r="U13">
+        <v>4</v>
+      </c>
+      <c r="V13" s="13">
+        <v>2</v>
+      </c>
+      <c r="W13">
+        <v>3</v>
+      </c>
+      <c r="X13" s="13">
+        <v>3</v>
+      </c>
+      <c r="Y13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B14" s="13">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14" s="13">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14" s="13">
+        <v>2</v>
+      </c>
+      <c r="G14">
+        <v>3</v>
+      </c>
+      <c r="H14" s="13">
+        <v>4</v>
+      </c>
+      <c r="I14">
+        <v>4</v>
+      </c>
+      <c r="J14" s="13">
+        <v>4</v>
+      </c>
+      <c r="K14">
+        <v>4</v>
+      </c>
+      <c r="L14" s="13">
+        <v>3</v>
+      </c>
+      <c r="M14">
+        <v>3</v>
+      </c>
+      <c r="N14" s="13">
+        <v>4</v>
+      </c>
+      <c r="O14">
+        <v>3</v>
+      </c>
+      <c r="P14" s="13">
+        <v>4</v>
+      </c>
+      <c r="Q14">
+        <v>4</v>
+      </c>
+      <c r="R14" s="13">
+        <v>4</v>
+      </c>
+      <c r="S14">
+        <v>3</v>
+      </c>
+      <c r="T14" s="13">
+        <v>3</v>
+      </c>
+      <c r="U14">
+        <v>4</v>
+      </c>
+      <c r="V14" s="13">
+        <v>4</v>
+      </c>
+      <c r="W14">
+        <v>4</v>
+      </c>
+      <c r="X14" s="13">
+        <v>5</v>
+      </c>
+      <c r="Y14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" s="13">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" s="13">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>2</v>
+      </c>
+      <c r="F15" s="13">
+        <v>4</v>
+      </c>
+      <c r="G15">
+        <v>5</v>
+      </c>
+      <c r="H15" s="13">
+        <v>4</v>
+      </c>
+      <c r="I15">
+        <v>4</v>
+      </c>
+      <c r="J15" s="13">
+        <v>2</v>
+      </c>
+      <c r="K15">
+        <v>5</v>
+      </c>
+      <c r="L15" s="13">
+        <v>2</v>
+      </c>
+      <c r="M15">
+        <v>5</v>
+      </c>
+      <c r="N15" s="13">
+        <v>5</v>
+      </c>
+      <c r="O15">
+        <v>5</v>
+      </c>
+      <c r="P15" s="13">
+        <v>5</v>
+      </c>
+      <c r="Q15">
+        <v>5</v>
+      </c>
+      <c r="R15" s="13">
+        <v>5</v>
+      </c>
+      <c r="S15">
+        <v>5</v>
+      </c>
+      <c r="T15" s="13">
+        <v>2</v>
+      </c>
+      <c r="U15">
+        <v>4</v>
+      </c>
+      <c r="V15" s="13">
+        <v>3</v>
+      </c>
+      <c r="W15">
+        <v>4</v>
+      </c>
+      <c r="X15" s="13">
+        <v>2</v>
+      </c>
+      <c r="Y15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B16" s="13">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>3</v>
+      </c>
+      <c r="D16" s="13">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16" s="13">
+        <v>2</v>
+      </c>
+      <c r="G16">
+        <v>2</v>
+      </c>
+      <c r="H16" s="13">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="J16" s="13">
+        <v>3</v>
+      </c>
+      <c r="K16">
+        <v>3</v>
+      </c>
+      <c r="L16" s="13">
+        <v>3</v>
+      </c>
+      <c r="M16">
+        <v>3</v>
+      </c>
+      <c r="N16" s="13">
+        <v>3</v>
+      </c>
+      <c r="O16">
+        <v>3</v>
+      </c>
+      <c r="P16" s="13">
+        <v>4</v>
+      </c>
+      <c r="Q16">
+        <v>4</v>
+      </c>
+      <c r="R16" s="13">
+        <v>4</v>
+      </c>
+      <c r="S16">
+        <v>4</v>
+      </c>
+      <c r="T16" s="13">
+        <v>3</v>
+      </c>
+      <c r="U16">
+        <v>2</v>
+      </c>
+      <c r="V16" s="13">
+        <v>3</v>
+      </c>
+      <c r="W16">
+        <v>4</v>
+      </c>
+      <c r="X16" s="13">
+        <v>4</v>
+      </c>
+      <c r="Y16">
+        <v>3</v>
+      </c>
       <c r="Z16" s="22"/>
       <c r="AA16" s="21"/>
       <c r="AB16" s="21"/>
@@ -1910,23 +2234,88 @@
       <c r="AD16" s="21"/>
       <c r="AE16" s="22"/>
     </row>
-    <row r="17" spans="3:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
-      <c r="K17" s="21"/>
-      <c r="R17" s="21"/>
-      <c r="S17" s="21"/>
-      <c r="T17" s="21"/>
-      <c r="U17" s="21"/>
+    <row r="17" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="13">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>4</v>
+      </c>
+      <c r="D17" s="13">
+        <v>3</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="F17" s="13">
+        <v>3</v>
+      </c>
+      <c r="G17">
+        <v>4</v>
+      </c>
+      <c r="H17" s="13">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>3</v>
+      </c>
+      <c r="J17" s="13">
+        <v>3</v>
+      </c>
+      <c r="K17">
+        <v>4</v>
+      </c>
+      <c r="L17" s="13">
+        <v>3</v>
+      </c>
+      <c r="M17">
+        <v>4</v>
+      </c>
+      <c r="N17" s="13">
+        <v>4</v>
+      </c>
+      <c r="O17">
+        <v>3</v>
+      </c>
+      <c r="P17" s="13">
+        <v>4</v>
+      </c>
+      <c r="Q17">
+        <v>3</v>
+      </c>
+      <c r="R17" s="13">
+        <v>4</v>
+      </c>
+      <c r="S17">
+        <v>3</v>
+      </c>
+      <c r="T17" s="13">
+        <v>3</v>
+      </c>
+      <c r="U17">
+        <v>4</v>
+      </c>
+      <c r="V17" s="13">
+        <v>3</v>
+      </c>
+      <c r="W17">
+        <v>3</v>
+      </c>
+      <c r="X17" s="13">
+        <v>3</v>
+      </c>
+      <c r="Y17">
+        <v>3</v>
+      </c>
       <c r="Z17" s="21"/>
       <c r="AA17" s="21"/>
       <c r="AE17" s="21"/>
     </row>
-    <row r="18" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="13"/>
       <c r="C18" s="20"/>
       <c r="E18" s="20"/>
       <c r="G18" s="20"/>
@@ -1942,14 +2331,8 @@
       <c r="AA18" s="21"/>
       <c r="AE18" s="21"/>
     </row>
-    <row r="19" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="21"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="21"/>
-      <c r="K19" s="21"/>
+    <row r="19" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
+      <c r="E19" s="26"/>
       <c r="R19" s="21"/>
       <c r="S19" s="21"/>
       <c r="T19" s="21"/>
@@ -1958,14 +2341,7 @@
       <c r="AA19" s="21"/>
       <c r="AE19" s="21"/>
     </row>
-    <row r="20" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="21"/>
-      <c r="K20" s="21"/>
+    <row r="20" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="R20" s="21"/>
       <c r="S20" s="21"/>
       <c r="T20" s="21"/>
@@ -1974,14 +2350,7 @@
       <c r="AA20" s="21"/>
       <c r="AE20" s="21"/>
     </row>
-    <row r="21" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
+    <row r="21" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="R21" s="21"/>
       <c r="S21" s="21"/>
       <c r="T21" s="21"/>
@@ -1990,14 +2359,7 @@
       <c r="AA21" s="21"/>
       <c r="AE21" s="21"/>
     </row>
-    <row r="22" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C22" s="20"/>
-      <c r="E22" s="20"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="21"/>
+    <row r="22" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="R22" s="21"/>
       <c r="S22" s="21"/>
       <c r="T22" s="21"/>
@@ -2006,14 +2368,7 @@
       <c r="AA22" s="21"/>
       <c r="AE22" s="21"/>
     </row>
-    <row r="23" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="C23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="21"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="21"/>
-      <c r="K23" s="21"/>
+    <row r="23" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="R23" s="21"/>
       <c r="S23" s="21"/>
       <c r="T23" s="21"/>
@@ -2022,7 +2377,7 @@
       <c r="AA23" s="21"/>
       <c r="AE23" s="21"/>
     </row>
-    <row r="24" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C24" s="20"/>
       <c r="E24" s="20"/>
       <c r="G24" s="20"/>
@@ -2038,7 +2393,7 @@
       <c r="AA24" s="21"/>
       <c r="AE24" s="21"/>
     </row>
-    <row r="25" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C25" s="20"/>
       <c r="E25" s="20"/>
       <c r="G25" s="20"/>
@@ -2054,7 +2409,7 @@
       <c r="AA25" s="21"/>
       <c r="AE25" s="21"/>
     </row>
-    <row r="26" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C26" s="20"/>
       <c r="E26" s="20"/>
       <c r="G26" s="20"/>
@@ -2070,7 +2425,7 @@
       <c r="AA26" s="21"/>
       <c r="AE26" s="21"/>
     </row>
-    <row r="27" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C27" s="20"/>
       <c r="E27" s="20"/>
       <c r="G27" s="20"/>
@@ -2162,18 +2517,18 @@
         <v>4</v>
       </c>
       <c r="D2" s="13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" s="20">
-        <v>3</v>
-      </c>
-      <c r="F2" s="25">
+        <v>4</v>
+      </c>
+      <c r="F2" s="24">
         <f>C2/B2</f>
         <v>0.8</v>
       </c>
-      <c r="G2" s="26">
+      <c r="G2" s="25">
         <f>E2/D2</f>
-        <v>0.6</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="H2" s="13"/>
       <c r="I2" s="20"/>
@@ -2210,12 +2565,12 @@
       <c r="E3" s="20">
         <v>4</v>
       </c>
-      <c r="F3" s="25">
-        <f t="shared" ref="F3:F12" si="0">C3/B3</f>
+      <c r="F3" s="24">
+        <f t="shared" ref="F3:F17" si="0">C3/B3</f>
         <v>1</v>
       </c>
-      <c r="G3" s="26">
-        <f t="shared" ref="G3:G12" si="1">E3/D3</f>
+      <c r="G3" s="25">
+        <f t="shared" ref="G3:G17" si="1">E3/D3</f>
         <v>0.66666666666666663</v>
       </c>
       <c r="H3" s="13"/>
@@ -2251,15 +2606,15 @@
         <v>5</v>
       </c>
       <c r="E4" s="20">
-        <v>1</v>
-      </c>
-      <c r="F4" s="25">
+        <v>2</v>
+      </c>
+      <c r="F4" s="24">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G4" s="26">
+      <c r="G4" s="25">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="H4" s="13"/>
       <c r="I4" s="20"/>
@@ -2291,18 +2646,18 @@
         <v>3</v>
       </c>
       <c r="D5" s="13">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E5" s="20">
-        <v>3</v>
-      </c>
-      <c r="F5" s="25">
+        <v>4</v>
+      </c>
+      <c r="F5" s="24">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G5" s="26">
+      <c r="G5" s="25">
         <f t="shared" si="1"/>
-        <v>0.6</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="H5" s="13"/>
       <c r="I5" s="20"/>
@@ -2339,11 +2694,11 @@
       <c r="E6" s="20">
         <v>4</v>
       </c>
-      <c r="F6" s="25">
+      <c r="F6" s="24">
         <f t="shared" si="0"/>
         <v>0.66666666666666663</v>
       </c>
-      <c r="G6" s="26">
+      <c r="G6" s="25">
         <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
@@ -2382,11 +2737,11 @@
       <c r="E7" s="20">
         <v>4</v>
       </c>
-      <c r="F7" s="25">
+      <c r="F7" s="24">
         <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
-      <c r="G7" s="26">
+      <c r="G7" s="25">
         <f t="shared" si="1"/>
         <v>0.5714285714285714</v>
       </c>
@@ -2425,11 +2780,11 @@
       <c r="E8" s="20">
         <v>3</v>
       </c>
-      <c r="F8" s="25">
+      <c r="F8" s="24">
         <f t="shared" si="0"/>
         <v>0.75</v>
       </c>
-      <c r="G8" s="26">
+      <c r="G8" s="25">
         <f t="shared" si="1"/>
         <v>0.6</v>
       </c>
@@ -2468,11 +2823,11 @@
       <c r="E9" s="20">
         <v>2</v>
       </c>
-      <c r="F9" s="25">
+      <c r="F9" s="24">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G9" s="26">
+      <c r="G9" s="25">
         <f t="shared" si="1"/>
         <v>0.66666666666666663</v>
       </c>
@@ -2506,18 +2861,18 @@
         <v>3</v>
       </c>
       <c r="D10" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E10" s="20">
-        <v>3</v>
-      </c>
-      <c r="F10" s="25">
+        <v>4</v>
+      </c>
+      <c r="F10" s="24">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G10" s="26">
+      <c r="G10" s="25">
         <f t="shared" si="1"/>
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="H10" s="13"/>
       <c r="I10" s="20"/>
@@ -2554,11 +2909,11 @@
       <c r="E11" s="20">
         <v>4</v>
       </c>
-      <c r="F11" s="25">
+      <c r="F11" s="24">
         <f t="shared" si="0"/>
         <v>0.66666666666666663</v>
       </c>
-      <c r="G11" s="26">
+      <c r="G11" s="25">
         <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
@@ -2597,11 +2952,11 @@
       <c r="E12" s="20">
         <v>4</v>
       </c>
-      <c r="F12" s="25">
+      <c r="F12" s="24">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G12" s="26">
+      <c r="G12" s="25">
         <f t="shared" si="1"/>
         <v>0.66666666666666663</v>
       </c>
@@ -2624,24 +2979,105 @@
       <c r="X12" s="13"/>
       <c r="Y12" s="20"/>
     </row>
+    <row r="13" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B13" s="13">
+        <v>5</v>
+      </c>
+      <c r="C13" s="20">
+        <v>3</v>
+      </c>
+      <c r="D13" s="13">
+        <v>8</v>
+      </c>
+      <c r="E13" s="20">
+        <v>5</v>
+      </c>
+      <c r="F13" s="24">
+        <f t="shared" si="0"/>
+        <v>0.6</v>
+      </c>
+      <c r="G13" s="25">
+        <f t="shared" si="1"/>
+        <v>0.625</v>
+      </c>
+    </row>
     <row r="14" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="23"/>
+      <c r="A14" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B14" s="13">
+        <v>5</v>
+      </c>
+      <c r="C14" s="13">
+        <v>3</v>
+      </c>
+      <c r="D14" s="13">
+        <v>8</v>
+      </c>
+      <c r="E14" s="13">
+        <v>7</v>
+      </c>
+      <c r="F14" s="23">
+        <f t="shared" si="0"/>
+        <v>0.6</v>
+      </c>
+      <c r="G14" s="25">
+        <f t="shared" si="1"/>
+        <v>0.875</v>
+      </c>
     </row>
     <row r="15" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
+      <c r="A15" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" s="13">
+        <v>3</v>
+      </c>
+      <c r="C15" s="13">
+        <v>3</v>
+      </c>
+      <c r="D15" s="13">
+        <v>6</v>
+      </c>
+      <c r="E15" s="13">
+        <v>5</v>
+      </c>
+      <c r="F15" s="24">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="G15" s="25">
+        <f t="shared" si="1"/>
+        <v>0.83333333333333337</v>
+      </c>
     </row>
     <row r="16" spans="1:31" ht="13" x14ac:dyDescent="0.3">
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
+      <c r="A16" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B16" s="13">
+        <v>5</v>
+      </c>
+      <c r="C16" s="13">
+        <v>4</v>
+      </c>
+      <c r="D16" s="13">
+        <v>7</v>
+      </c>
+      <c r="E16" s="13">
+        <v>4</v>
+      </c>
+      <c r="F16" s="24">
+        <f t="shared" si="0"/>
+        <v>0.8</v>
+      </c>
+      <c r="G16" s="24">
+        <f t="shared" si="1"/>
+        <v>0.5714285714285714</v>
+      </c>
       <c r="H16" s="22"/>
       <c r="I16" s="22"/>
       <c r="J16" s="21"/>
@@ -2667,10 +3103,30 @@
       <c r="AD16" s="21"/>
       <c r="AE16" s="22"/>
     </row>
-    <row r="17" spans="3:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="G17" s="20"/>
+    <row r="17" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="13">
+        <v>6</v>
+      </c>
+      <c r="C17" s="13">
+        <v>3</v>
+      </c>
+      <c r="D17" s="13">
+        <v>5</v>
+      </c>
+      <c r="E17" s="13">
+        <v>4</v>
+      </c>
+      <c r="F17" s="24">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="G17" s="24">
+        <f t="shared" si="1"/>
+        <v>0.8</v>
+      </c>
       <c r="H17" s="21"/>
       <c r="I17" s="21"/>
       <c r="J17" s="21"/>
@@ -2683,7 +3139,7 @@
       <c r="AA17" s="21"/>
       <c r="AE17" s="21"/>
     </row>
-    <row r="18" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C18" s="20"/>
       <c r="E18" s="20"/>
       <c r="G18" s="20"/>
@@ -2699,9 +3155,9 @@
       <c r="AA18" s="21"/>
       <c r="AE18" s="21"/>
     </row>
-    <row r="19" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C19" s="20"/>
-      <c r="E19" s="20"/>
+      <c r="E19" s="27"/>
       <c r="G19" s="20"/>
       <c r="H19" s="21"/>
       <c r="I19" s="21"/>
@@ -2715,7 +3171,7 @@
       <c r="AA19" s="21"/>
       <c r="AE19" s="21"/>
     </row>
-    <row r="20" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C20" s="20"/>
       <c r="E20" s="20"/>
       <c r="G20" s="20"/>
@@ -2731,7 +3187,7 @@
       <c r="AA20" s="21"/>
       <c r="AE20" s="21"/>
     </row>
-    <row r="21" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C21" s="20"/>
       <c r="E21" s="20"/>
       <c r="G21" s="20"/>
@@ -2747,7 +3203,7 @@
       <c r="AA21" s="21"/>
       <c r="AE21" s="21"/>
     </row>
-    <row r="22" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C22" s="20"/>
       <c r="E22" s="20"/>
       <c r="G22" s="20"/>
@@ -2763,7 +3219,7 @@
       <c r="AA22" s="21"/>
       <c r="AE22" s="21"/>
     </row>
-    <row r="23" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C23" s="20"/>
       <c r="E23" s="20"/>
       <c r="G23" s="20"/>
@@ -2779,7 +3235,7 @@
       <c r="AA23" s="21"/>
       <c r="AE23" s="21"/>
     </row>
-    <row r="24" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C24" s="20"/>
       <c r="E24" s="20"/>
       <c r="G24" s="20"/>
@@ -2795,7 +3251,7 @@
       <c r="AA24" s="21"/>
       <c r="AE24" s="21"/>
     </row>
-    <row r="25" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C25" s="20"/>
       <c r="E25" s="20"/>
       <c r="G25" s="20"/>
@@ -2811,7 +3267,7 @@
       <c r="AA25" s="21"/>
       <c r="AE25" s="21"/>
     </row>
-    <row r="26" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C26" s="20"/>
       <c r="E26" s="20"/>
       <c r="G26" s="20"/>
@@ -2827,7 +3283,7 @@
       <c r="AA26" s="21"/>
       <c r="AE26" s="21"/>
     </row>
-    <row r="27" spans="3:31" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:31" ht="12.5" x14ac:dyDescent="0.25">
       <c r="C27" s="20"/>
       <c r="E27" s="20"/>
       <c r="G27" s="20"/>
@@ -2844,6 +3300,7 @@
       <c r="AE27" s="21"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>